<commit_message>
chore(data): normalize Gartner card list
Strip stray whitespace and fix 'Ex' casing in names and card types. Fold the
Yanmega ex #206 row on the Ascended Heroes tab into the Destined Rivals #206
row (3 + 1), correct Arbok ex 185/162 to 185/165, and drop the Yanmega #228
link that pointed at the #206 product.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/data-files/gartner-it-symposium-2026/TCG Search Raw List - Gartner IT Symposium 2026.xlsx
+++ b/data/data-files/gartner-it-symposium-2026/TCG Search Raw List - Gartner IT Symposium 2026.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D2" s="19" t="n">
@@ -738,7 +738,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss's Orders  </t>
+          <t>Boss's Orders</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
@@ -1263,7 +1263,7 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Canari </t>
+          <t>Canari</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mega Gengar ex </t>
+          <t>Mega Gengar ex</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
@@ -1438,7 +1438,7 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lillie's Clefairy ex </t>
+          <t>Lillie's Clefairy ex</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mega Audino ex </t>
+          <t>Mega Audino ex</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1681,39 +1681,15 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Yanmega ex</t>
-        </is>
-      </c>
-      <c r="B34" s="23" t="inlineStr">
-        <is>
-          <t>206/182</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
-        <is>
-          <t>Ultra Rare</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="8" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="F34" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="I34" s="12" t="b">
-        <v>1</v>
-      </c>
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="23" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="12" t="n"/>
+      <c r="I34" s="12" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -1788,7 +1764,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mega Feraligatr ex </t>
+          <t>Mega Feraligatr ex</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
@@ -1963,7 +1939,7 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black Belt's Training </t>
+          <t>Black Belt's Training</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
@@ -1998,7 +1974,7 @@
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mega Audino ex </t>
+          <t>Mega Audino ex</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2418,7 +2394,7 @@
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>Ethan's Ho-Oh Ex</t>
+          <t>Ethan's Ho-Oh ex</t>
         </is>
       </c>
       <c r="B55" s="17" t="inlineStr">
@@ -2663,7 +2639,7 @@
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>Cinderace Ex</t>
+          <t>Cinderace ex</t>
         </is>
       </c>
       <c r="B62" s="17" t="inlineStr">
@@ -5108,41 +5084,40 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5294,7 +5269,7 @@
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D3" s="41" t="n">
@@ -5396,7 +5371,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D5" s="41" t="n">
@@ -5539,7 +5514,7 @@
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Team Rocket's Giovanni </t>
+          <t>Team Rocket's Giovanni</t>
         </is>
       </c>
       <c r="B8" s="36" t="inlineStr">
@@ -5651,7 +5626,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D10" s="41" t="n">
@@ -6212,7 +6187,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D21" s="44" t="n">
@@ -6263,7 +6238,7 @@
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D22" s="41" t="n">
@@ -6304,7 +6279,7 @@
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Ethan's Ho-Oh Ex</t>
+          <t>Ethan's Ho-Oh ex</t>
         </is>
       </c>
       <c r="B23" s="27" t="inlineStr">
@@ -6406,7 +6381,7 @@
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Team Rocket's Giovanni </t>
+          <t>Team Rocket's Giovanni</t>
         </is>
       </c>
       <c r="B25" s="36" t="inlineStr">
@@ -6967,7 +6942,7 @@
     <row r="36">
       <c r="A36" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Team Rocket's Archer </t>
+          <t>Team Rocket's Archer</t>
         </is>
       </c>
       <c r="B36" s="36" t="inlineStr">
@@ -7032,7 +7007,7 @@
         </is>
       </c>
       <c r="D37" s="41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="18" t="n">
         <v>1.57</v>
@@ -7120,7 +7095,7 @@
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>Dondozo Ex</t>
+          <t>Dondozo ex</t>
         </is>
       </c>
       <c r="B39" s="27" t="inlineStr">
@@ -7428,7 +7403,7 @@
     <row r="45">
       <c r="A45" s="26" t="inlineStr">
         <is>
-          <t>Ethan's Ho-Oh Ex</t>
+          <t>Ethan's Ho-Oh ex</t>
         </is>
       </c>
       <c r="B45" s="27" t="inlineStr">
@@ -26953,47 +26928,46 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27337,7 +27311,7 @@
     <row r="7">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulbasaur </t>
+          <t>Bulbasaur</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
@@ -27908,7 +27882,7 @@
       </c>
       <c r="C18" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D18" s="41" t="n">
@@ -28413,7 +28387,7 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>185/162</t>
+          <t>185/165</t>
         </is>
       </c>
       <c r="C28" s="42" t="inlineStr">
@@ -52453,7 +52427,7 @@
       </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gold </t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="D2" s="12" t="n">

</xml_diff>